<commit_message>
KPI actualizado 2026-07-23 15:14 UTC
</commit_message>
<xml_diff>
--- a/data/50001580- CIA. RIO MINERALES.xlsx
+++ b/data/50001580- CIA. RIO MINERALES.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="334">
   <si>
     <t>50001580- "CIA. RIO MINERALES"</t>
   </si>
@@ -250,6 +250,14 @@
   </si>
   <si>
     <t>1216788147959225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Ficha técnica ventilador
+    Hoja de datos motor
+    Plano Montaje
+    Plano Cimentación
+    Manual de Operación y Servicio
+</t>
   </si>
   <si>
     <t>Ingenieria Jefe de proyecto:,Plano Preliminar OT4378</t>
@@ -1857,7 +1865,7 @@
         <v>46226.571240590274</v>
       </c>
       <c r="D7" s="9">
-        <v>46226.571264432874</v>
+        <v>46226.572476099536</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>38</v>
@@ -2262,9 +2270,11 @@
       <c r="B14" s="5">
         <v>46225.58085679398</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46226.57610013889</v>
+      </c>
       <c r="D14" s="5">
-        <v>46225.59597591435</v>
+        <v>46226.576112442126</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>66</v>
@@ -2299,8 +2309,12 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
+      <c r="T14" s="6">
+        <v>1</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
@@ -2309,9 +2323,11 @@
       <c r="B15" s="9">
         <v>46225.58095215278</v>
       </c>
-      <c r="C15" s="10"/>
+      <c r="C15" s="9">
+        <v>46226.576076365745</v>
+      </c>
       <c r="D15" s="9">
-        <v>46226.571272754634</v>
+        <v>46226.57609552083</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>67</v>
@@ -2335,7 +2351,7 @@
         <v>26</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>26</v>
+        <v>69</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>26</v>
@@ -2347,7 +2363,7 @@
         <v>38</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="9">
         <v>46227</v>
@@ -2359,15 +2375,15 @@
         <v>33</v>
       </c>
       <c r="T15" s="10">
-        <v>0</v>
-      </c>
-      <c r="U15" s="11" t="s">
-        <v>52</v>
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46225.580861423616</v>
@@ -2377,7 +2393,7 @@
         <v>46225.59611458333</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>25</v>
@@ -2401,7 +2417,7 @@
         <v>26</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P16" s="6" t="s">
         <v>26</v>
@@ -2414,7 +2430,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B17" s="9">
         <v>46225.580958923616</v>
@@ -2424,16 +2440,16 @@
         <v>46226.57127291667</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I17" s="9">
         <v>46226</v>
@@ -2451,13 +2467,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="9">
         <v>46227</v>
@@ -2477,7 +2493,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B18" s="5">
         <v>46225.58096494213</v>
@@ -2487,16 +2503,16 @@
         <v>46226.57127292824</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I18" s="5">
         <v>46226</v>
@@ -2514,13 +2530,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>38</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q18" s="5">
         <v>46227</v>
@@ -2540,7 +2556,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9">
         <v>46225.58097109954</v>
@@ -2550,16 +2566,16 @@
         <v>46226.571272870366</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I19" s="9">
         <v>46226</v>
@@ -2577,13 +2593,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="9">
         <v>46227</v>
@@ -2603,7 +2619,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" s="5">
         <v>46225.58086628473</v>
@@ -2613,7 +2629,7 @@
         <v>46225.59619578704</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>25</v>
@@ -2637,7 +2653,7 @@
         <v>26</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>26</v>
@@ -2650,7 +2666,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21" s="9">
         <v>46225.580978240745</v>
@@ -2660,16 +2676,16 @@
         <v>46225.61247136574</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I21" s="9">
         <v>46245</v>
@@ -2687,13 +2703,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q21" s="9">
         <v>46246</v>
@@ -2713,7 +2729,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B22" s="5">
         <v>46225.5809840625</v>
@@ -2723,16 +2739,16 @@
         <v>46225.612467824074</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I22" s="5">
         <v>46245</v>
@@ -2750,13 +2766,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q22" s="5">
         <v>46246</v>
@@ -2776,7 +2792,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B23" s="9">
         <v>46225.58098827546</v>
@@ -2786,16 +2802,16 @@
         <v>46225.612464756945</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I23" s="9">
         <v>46245</v>
@@ -2813,13 +2829,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q23" s="9">
         <v>46246</v>
@@ -2839,7 +2855,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B24" s="5">
         <v>46225.58100011574</v>
@@ -2849,16 +2865,16 @@
         <v>46225.61246184028</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I24" s="5">
         <v>46245</v>
@@ -2876,13 +2892,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q24" s="5">
         <v>46246</v>
@@ -2902,7 +2918,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B25" s="9">
         <v>46225.59619364583</v>
@@ -2912,16 +2928,16 @@
         <v>46225.61245637732</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I25" s="9">
         <v>46231</v>
@@ -2939,13 +2955,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>48</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q25" s="9">
         <v>46232</v>
@@ -2965,7 +2981,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B26" s="5">
         <v>46225.58087085648</v>
@@ -2975,7 +2991,7 @@
         <v>46225.596821886575</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>25</v>
@@ -2999,7 +3015,7 @@
         <v>26</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>26</v>
@@ -3012,7 +3028,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B27" s="9">
         <v>46225.58100560185</v>
@@ -3022,16 +3038,16 @@
         <v>46225.61255763889</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I27" s="9">
         <v>46247</v>
@@ -3049,13 +3065,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q27" s="9">
         <v>46259</v>
@@ -3075,7 +3091,7 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B28" s="5">
         <v>46225.58101144676</v>
@@ -3085,16 +3101,16 @@
         <v>46225.61262662037</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I28" s="5">
         <v>46247</v>
@@ -3112,13 +3128,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3134,7 +3150,7 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B29" s="9">
         <v>46225.581017233795</v>
@@ -3144,16 +3160,16 @@
         <v>46225.61262351852</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I29" s="9">
         <v>46251</v>
@@ -3171,13 +3187,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q29" s="10"/>
       <c r="R29" s="10"/>
@@ -3193,7 +3209,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B30" s="5">
         <v>46225.58102277778</v>
@@ -3203,16 +3219,16 @@
         <v>46225.61255446759</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I30" s="5">
         <v>46247</v>
@@ -3230,10 +3246,10 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>26</v>
@@ -3256,7 +3272,7 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B31" s="9">
         <v>46225.58102737268</v>
@@ -3266,16 +3282,16 @@
         <v>46225.61269579861</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I31" s="9">
         <v>46247</v>
@@ -3293,13 +3309,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
@@ -3309,7 +3325,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B32" s="5">
         <v>46225.581032222224</v>
@@ -3319,16 +3335,16 @@
         <v>46225.612692442126</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I32" s="5">
         <v>46251</v>
@@ -3346,13 +3362,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3362,7 +3378,7 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B33" s="9">
         <v>46225.581037199074</v>
@@ -3372,16 +3388,16 @@
         <v>46225.61279568287</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I33" s="9">
         <v>46247</v>
@@ -3399,10 +3415,10 @@
         <v>26</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>26</v>
@@ -3425,7 +3441,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B34" s="5">
         <v>46225.58104158565</v>
@@ -3435,16 +3451,16 @@
         <v>46225.61298453704</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I34" s="5">
         <v>46247</v>
@@ -3462,13 +3478,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3478,7 +3494,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B35" s="9">
         <v>46225.5810464699</v>
@@ -3488,16 +3504,16 @@
         <v>46225.61298125</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I35" s="9">
         <v>46251</v>
@@ -3515,13 +3531,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
@@ -3531,7 +3547,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B36" s="5">
         <v>46225.58105121528</v>
@@ -3541,16 +3557,16 @@
         <v>46225.61316422454</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I36" s="5">
         <v>46247</v>
@@ -3568,10 +3584,10 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3594,7 +3610,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B37" s="9">
         <v>46225.58109630787</v>
@@ -3604,16 +3620,16 @@
         <v>46225.613052245375</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I37" s="9">
         <v>46247</v>
@@ -3631,13 +3647,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3647,7 +3663,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B38" s="5">
         <v>46225.58110178241</v>
@@ -3657,16 +3673,16 @@
         <v>46225.613047719904</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I38" s="5">
         <v>46258</v>
@@ -3684,13 +3700,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3700,7 +3716,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B39" s="9">
         <v>46225.58110600694</v>
@@ -3710,16 +3726,16 @@
         <v>46225.613129363424</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I39" s="9">
         <v>46289</v>
@@ -3737,13 +3753,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P39" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q39" s="10"/>
       <c r="R39" s="10"/>
@@ -3753,7 +3769,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B40" s="5">
         <v>46225.59682005787</v>
@@ -3763,16 +3779,16 @@
         <v>46225.6133383912</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I40" s="5">
         <v>46233</v>
@@ -3790,10 +3806,10 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>26</v>
@@ -3816,7 +3832,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" s="9">
         <v>46225.59686481481</v>
@@ -3826,16 +3842,16 @@
         <v>46225.613313634254</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I41" s="9">
         <v>46233</v>
@@ -3853,13 +3869,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -3869,7 +3885,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B42" s="5">
         <v>46225.59692966435</v>
@@ -3879,16 +3895,16 @@
         <v>46225.613310636574</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I42" s="5">
         <v>46244</v>
@@ -3906,13 +3922,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
@@ -3922,7 +3938,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B43" s="9">
         <v>46225.58111748843</v>
@@ -3932,7 +3948,7 @@
         <v>46225.589328946764</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>25</v>
@@ -3956,7 +3972,7 @@
         <v>26</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -3969,26 +3985,26 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B44" s="5">
         <v>46225.58112127315</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46225.61343114583</v>
+        <v>46226.57609570602</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I44" s="5">
         <v>46230</v>
@@ -4006,13 +4022,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>67</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q44" s="5">
         <v>46234</v>
@@ -4026,13 +4042,13 @@
       <c r="T44" s="6">
         <v>0</v>
       </c>
-      <c r="U44" s="12" t="s">
-        <v>58</v>
+      <c r="U44" s="11" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B45" s="9">
         <v>46225.58112643519</v>
@@ -4042,16 +4058,16 @@
         <v>46225.613428275465</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I45" s="9">
         <v>46237</v>
@@ -4069,13 +4085,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Q45" s="9">
         <v>46241</v>
@@ -4095,7 +4111,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B46" s="5">
         <v>46225.58113097222</v>
@@ -4105,16 +4121,16 @@
         <v>46225.61342412037</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I46" s="5">
         <v>46244</v>
@@ -4132,13 +4148,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q46" s="5">
         <v>46244</v>
@@ -4158,7 +4174,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B47" s="9">
         <v>46225.58114445602</v>
@@ -4168,16 +4184,16 @@
         <v>46225.61347256944</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I47" s="9">
         <v>46290</v>
@@ -4195,13 +4211,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q47" s="9">
         <v>46290</v>
@@ -4221,7 +4237,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B48" s="5">
         <v>46225.58114871528</v>
@@ -4231,16 +4247,16 @@
         <v>46225.61551950232</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I48" s="5">
         <v>46290</v>
@@ -4258,13 +4274,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
@@ -4274,7 +4290,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B49" s="9">
         <v>46225.58115283565</v>
@@ -4284,16 +4300,16 @@
         <v>46225.615519513885</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I49" s="9">
         <v>46290</v>
@@ -4311,13 +4327,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q49" s="10"/>
       <c r="R49" s="10"/>
@@ -4327,7 +4343,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B50" s="5">
         <v>46225.581171631944</v>
@@ -4337,7 +4353,7 @@
         <v>46225.59181146991</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>25</v>
@@ -4361,7 +4377,7 @@
         <v>26</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4374,7 +4390,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B51" s="9">
         <v>46225.58117489584</v>
@@ -4384,16 +4400,16 @@
         <v>46225.61367097222</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I51" s="9">
         <v>46260</v>
@@ -4411,13 +4427,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Q51" s="9">
         <v>46260</v>
@@ -4437,7 +4453,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B52" s="5">
         <v>46225.58118028935</v>
@@ -4447,16 +4463,16 @@
         <v>46225.613667349535</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I52" s="5">
         <v>46260</v>
@@ -4474,13 +4490,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="Q52" s="5">
         <v>46260</v>
@@ -4500,7 +4516,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B53" s="9">
         <v>46225.58118576389</v>
@@ -4510,16 +4526,16 @@
         <v>46225.61366387732</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I53" s="9">
         <v>46260</v>
@@ -4537,13 +4553,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="Q53" s="9">
         <v>46260</v>
@@ -4563,7 +4579,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B54" s="5">
         <v>46225.58119107639</v>
@@ -4573,16 +4589,16 @@
         <v>46225.61417395833</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I54" s="5">
         <v>46261</v>
@@ -4600,13 +4616,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q54" s="5">
         <v>46261</v>
@@ -4626,7 +4642,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B55" s="9">
         <v>46225.58119642361</v>
@@ -4636,16 +4652,16 @@
         <v>46225.61417104167</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I55" s="9">
         <v>46261</v>
@@ -4663,13 +4679,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="Q55" s="9">
         <v>46261</v>
@@ -4689,7 +4705,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B56" s="5">
         <v>46225.581201678244</v>
@@ -4699,16 +4715,16 @@
         <v>46225.61416773148</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I56" s="5">
         <v>46261</v>
@@ -4726,13 +4742,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q56" s="5">
         <v>46261</v>
@@ -4752,7 +4768,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B57" s="9">
         <v>46225.58120702546</v>
@@ -4762,7 +4778,7 @@
         <v>46225.59190644676</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>25</v>
@@ -4786,7 +4802,7 @@
         <v>26</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P57" s="10" t="s">
         <v>26</v>
@@ -4799,7 +4815,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B58" s="5">
         <v>46225.58121010417</v>
@@ -4809,16 +4825,16 @@
         <v>46225.6142333912</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I58" s="5">
         <v>46262</v>
@@ -4836,13 +4852,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q58" s="5">
         <v>46266</v>
@@ -4862,7 +4878,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B59" s="9">
         <v>46225.581215474536</v>
@@ -4872,16 +4888,16 @@
         <v>46225.61435628472</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I59" s="9">
         <v>46267</v>
@@ -4899,13 +4915,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q59" s="9">
         <v>46273</v>
@@ -4925,7 +4941,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B60" s="5">
         <v>46225.581219618056</v>
@@ -4935,16 +4951,16 @@
         <v>46225.614318611115</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I60" s="5">
         <v>46267</v>
@@ -4962,13 +4978,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
@@ -4978,7 +4994,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B61" s="9">
         <v>46225.58123596065</v>
@@ -4988,16 +5004,16 @@
         <v>46225.61431550926</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I61" s="9">
         <v>46267</v>
@@ -5015,13 +5031,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q61" s="10"/>
       <c r="R61" s="10"/>
@@ -5031,7 +5047,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B62" s="5">
         <v>46225.58129219907</v>
@@ -5041,16 +5057,16 @@
         <v>46225.61447392361</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I62" s="5">
         <v>46274</v>
@@ -5068,13 +5084,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q62" s="5">
         <v>46274</v>
@@ -5094,7 +5110,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B63" s="9">
         <v>46225.58129802083</v>
@@ -5104,16 +5120,16 @@
         <v>46225.61443357639</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I63" s="10"/>
       <c r="J63" s="9">
@@ -5129,13 +5145,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Q63" s="10"/>
       <c r="R63" s="10"/>
@@ -5145,7 +5161,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B64" s="5">
         <v>46225.581304374995</v>
@@ -5155,16 +5171,16 @@
         <v>46225.61443052083</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
@@ -5180,13 +5196,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5196,7 +5212,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B65" s="9">
         <v>46225.58131015046</v>
@@ -5206,7 +5222,7 @@
         <v>46225.59759329861</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>25</v>
@@ -5230,7 +5246,7 @@
         <v>26</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="P65" s="10" t="s">
         <v>26</v>
@@ -5243,7 +5259,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B66" s="5">
         <v>46225.58131376158</v>
@@ -5253,16 +5269,16 @@
         <v>46225.61459215278</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I66" s="5">
         <v>46230</v>
@@ -5280,13 +5296,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Q66" s="5">
         <v>46231</v>
@@ -5306,7 +5322,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B67" s="9">
         <v>46225.58131929398</v>
@@ -5316,16 +5332,16 @@
         <v>46225.61459149305</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I67" s="9">
         <v>46230</v>
@@ -5343,13 +5359,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Q67" s="9">
         <v>46231</v>
@@ -5369,7 +5385,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B68" s="5">
         <v>46225.58132505787</v>
@@ -5379,16 +5395,16 @@
         <v>46225.61459082176</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I68" s="5">
         <v>46230</v>
@@ -5406,13 +5422,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Q68" s="5">
         <v>46231</v>
@@ -5432,7 +5448,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B69" s="9">
         <v>46225.597591134254</v>
@@ -5448,10 +5464,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I69" s="9">
         <v>46293</v>
@@ -5469,10 +5485,10 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P69" s="10" t="s">
         <v>57</v>
@@ -5495,7 +5511,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B70" s="5">
         <v>46225.58133054398</v>
@@ -5505,7 +5521,7 @@
         <v>46225.59299179398</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>25</v>
@@ -5529,7 +5545,7 @@
         <v>26</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>26</v>
@@ -5542,7 +5558,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B71" s="9">
         <v>46225.58133395833</v>
@@ -5552,16 +5568,16 @@
         <v>46225.614863599534</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I71" s="9">
         <v>46275</v>
@@ -5579,13 +5595,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q71" s="9">
         <v>46281</v>
@@ -5605,7 +5621,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B72" s="5">
         <v>46225.58133853009</v>
@@ -5615,16 +5631,16 @@
         <v>46225.61483068287</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I72" s="5">
         <v>46275</v>
@@ -5642,13 +5658,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="Q72" s="6"/>
       <c r="R72" s="6"/>
@@ -5658,7 +5674,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B73" s="9">
         <v>46225.58134314815</v>
@@ -5668,16 +5684,16 @@
         <v>46225.61482673611</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I73" s="9">
         <v>46275</v>
@@ -5695,13 +5711,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q73" s="10"/>
       <c r="R73" s="10"/>
@@ -5711,7 +5727,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B74" s="5">
         <v>46225.58134744213</v>
@@ -5721,16 +5737,16 @@
         <v>46225.61499751157</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I74" s="5">
         <v>46286</v>
@@ -5748,13 +5764,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q74" s="5">
         <v>46286</v>
@@ -5774,7 +5790,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B75" s="9">
         <v>46225.581351932866</v>
@@ -5784,16 +5800,16 @@
         <v>46225.61504185185</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I75" s="9">
         <v>46286</v>
@@ -5811,13 +5827,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q75" s="10"/>
       <c r="R75" s="10"/>
@@ -5827,7 +5843,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B76" s="5">
         <v>46225.58135922454</v>
@@ -5837,16 +5853,16 @@
         <v>46225.615038819444</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I76" s="5">
         <v>46286</v>
@@ -5864,13 +5880,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -5880,7 +5896,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B77" s="9">
         <v>46225.5813728588</v>
@@ -5890,16 +5906,16 @@
         <v>46225.61522760417</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I77" s="9">
         <v>46287</v>
@@ -5917,13 +5933,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q77" s="9">
         <v>46287</v>
@@ -5943,7 +5959,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B78" s="5">
         <v>46225.58137722222</v>
@@ -5953,16 +5969,16 @@
         <v>46225.61518142361</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="5">
@@ -5978,13 +5994,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Q78" s="6"/>
       <c r="R78" s="6"/>
@@ -5994,7 +6010,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B79" s="9">
         <v>46225.58138231482</v>
@@ -6004,16 +6020,16 @@
         <v>46225.615182291665</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6029,13 +6045,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Q79" s="10"/>
       <c r="R79" s="10"/>
@@ -6045,7 +6061,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B80" s="5">
         <v>46225.58138733797</v>
@@ -6055,16 +6071,16 @@
         <v>46225.61538164352</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I80" s="5">
         <v>46288</v>
@@ -6082,13 +6098,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q80" s="5">
         <v>46288</v>
@@ -6108,7 +6124,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B81" s="9">
         <v>46225.58139180556</v>
@@ -6118,16 +6134,16 @@
         <v>46225.61534716435</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I81" s="9">
         <v>46288</v>
@@ -6145,13 +6161,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q81" s="10"/>
       <c r="R81" s="10"/>
@@ -6161,7 +6177,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B82" s="5">
         <v>46225.58139752314</v>
@@ -6171,16 +6187,16 @@
         <v>46225.615343854166</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I82" s="5">
         <v>46288</v>
@@ -6198,13 +6214,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6214,7 +6230,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B83" s="9">
         <v>46225.58140275463</v>
@@ -6224,16 +6240,16 @@
         <v>46225.61555996528</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I83" s="9">
         <v>46289</v>
@@ -6251,13 +6267,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q83" s="9">
         <v>46289</v>
@@ -6277,7 +6293,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B84" s="5">
         <v>46225.581407488426</v>
@@ -6287,16 +6303,16 @@
         <v>46225.61551967592</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="5">
@@ -6312,13 +6328,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q84" s="6"/>
       <c r="R84" s="6"/>
@@ -6328,7 +6344,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B85" s="9">
         <v>46225.581414988425</v>
@@ -6338,16 +6354,16 @@
         <v>46225.61552056713</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="9">
@@ -6363,13 +6379,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q85" s="10"/>
       <c r="R85" s="10"/>
@@ -6379,7 +6395,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B86" s="5">
         <v>46225.58145953703</v>
@@ -6389,7 +6405,7 @@
         <v>46225.61568145834</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6414,13 +6430,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q86" s="5">
         <v>46293</v>
@@ -6440,7 +6456,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B87" s="9">
         <v>46225.58146568287</v>
@@ -6450,16 +6466,16 @@
         <v>46225.61568175926</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I87" s="9">
         <v>46293</v>
@@ -6477,13 +6493,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6493,7 +6509,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B88" s="5">
         <v>46225.58147099537</v>
@@ -6503,16 +6519,16 @@
         <v>46225.615682592594</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I88" s="5">
         <v>46293</v>
@@ -6530,13 +6546,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q88" s="6"/>
       <c r="R88" s="6"/>
@@ -6546,7 +6562,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B89" s="9">
         <v>46225.58147606481</v>
@@ -6556,7 +6572,7 @@
         <v>46225.60367008102</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>25</v>
@@ -6580,7 +6596,7 @@
         <v>26</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P89" s="10" t="s">
         <v>26</v>
@@ -6593,7 +6609,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B90" s="5">
         <v>46225.58147990741</v>
@@ -6603,16 +6619,16 @@
         <v>46225.615814467594</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I90" s="5">
         <v>46301</v>
@@ -6630,13 +6646,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q90" s="5">
         <v>46301</v>
@@ -6656,7 +6672,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B91" s="9">
         <v>46225.58148496528</v>
@@ -6666,16 +6682,16 @@
         <v>46225.61578579861</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="9">
@@ -6691,13 +6707,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q91" s="10"/>
       <c r="R91" s="10"/>
@@ -6707,7 +6723,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B92" s="5">
         <v>46225.58148953704</v>
@@ -6717,16 +6733,16 @@
         <v>46225.61578274306</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I92" s="5">
         <v>46301</v>
@@ -6744,13 +6760,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -6760,7 +6776,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B93" s="9">
         <v>46225.6055390625</v>
@@ -6770,16 +6786,16 @@
         <v>46225.61577960648</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="9">
@@ -6795,13 +6811,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O93" s="10" t="s">
         <v>60</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -6811,7 +6827,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B94" s="5">
         <v>46225.605553333335</v>
@@ -6821,16 +6837,16 @@
         <v>46225.61577443287</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="5">
@@ -6846,13 +6862,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>64</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q94" s="6"/>
       <c r="R94" s="6"/>
@@ -6862,7 +6878,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B95" s="9">
         <v>46225.581494178245</v>
@@ -6872,16 +6888,16 @@
         <v>46225.61592174768</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="9">
@@ -6897,10 +6913,10 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P95" s="10" t="s">
         <v>26</v>
@@ -6923,7 +6939,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B96" s="5">
         <v>46225.5814984375</v>
@@ -6933,16 +6949,16 @@
         <v>46225.615894421295</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I96" s="5">
         <v>46302</v>
@@ -6960,13 +6976,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -6976,7 +6992,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B97" s="9">
         <v>46225.58150320602</v>
@@ -6986,16 +7002,16 @@
         <v>46225.61589104167</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I97" s="9">
         <v>46302</v>
@@ -7013,13 +7029,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7029,7 +7045,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B98" s="5">
         <v>46225.60673211806</v>
@@ -7039,16 +7055,16 @@
         <v>46225.615888125</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I98" s="5">
         <v>46302</v>
@@ -7066,13 +7082,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -7082,7 +7098,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B99" s="9">
         <v>46225.60674163194</v>
@@ -7092,16 +7108,16 @@
         <v>46225.61588293982</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I99" s="9">
         <v>46302</v>
@@ -7119,13 +7135,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="Q99" s="10"/>
       <c r="R99" s="10"/>
@@ -7135,7 +7151,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B100" s="5">
         <v>46225.58150777778</v>
@@ -7145,16 +7161,16 @@
         <v>46225.61603868056</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I100" s="5">
         <v>46303</v>
@@ -7172,13 +7188,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Q100" s="5">
         <v>46303</v>
@@ -7198,7 +7214,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B101" s="9">
         <v>46225.58151239583</v>
@@ -7208,16 +7224,16 @@
         <v>46225.61600570602</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H101" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="9">
@@ -7233,13 +7249,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q101" s="10"/>
       <c r="R101" s="10"/>
@@ -7249,7 +7265,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B102" s="5">
         <v>46225.58151694444</v>
@@ -7259,16 +7275,16 @@
         <v>46225.61600274306</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="5">
@@ -7284,13 +7300,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7300,7 +7316,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B103" s="9">
         <v>46225.606768564816</v>
@@ -7310,16 +7326,16 @@
         <v>46225.615999965274</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I103" s="9">
         <v>46303</v>
@@ -7337,13 +7353,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Q103" s="10"/>
       <c r="R103" s="10"/>
@@ -7353,7 +7369,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B104" s="5">
         <v>46225.606777395835</v>
@@ -7363,16 +7379,16 @@
         <v>46225.61599523148</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I104" s="5">
         <v>46303</v>
@@ -7390,13 +7406,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Q104" s="6"/>
       <c r="R104" s="6"/>
@@ -7406,7 +7422,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B105" s="9">
         <v>46225.581521562504</v>
@@ -7416,16 +7432,16 @@
         <v>46225.61624585648</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I105" s="9">
         <v>46304</v>
@@ -7443,13 +7459,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q105" s="9">
         <v>46304</v>
@@ -7469,7 +7485,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B106" s="5">
         <v>46225.58152704861</v>
@@ -7479,16 +7495,16 @@
         <v>46225.61621090278</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I106" s="6"/>
       <c r="J106" s="5">
@@ -7504,13 +7520,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7520,7 +7536,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B107" s="9">
         <v>46225.58153157408</v>
@@ -7530,16 +7546,16 @@
         <v>46225.61620709491</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H107" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I107" s="10"/>
       <c r="J107" s="9">
@@ -7555,13 +7571,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q107" s="10"/>
       <c r="R107" s="10"/>
@@ -7571,7 +7587,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B108" s="5">
         <v>46225.60680554398</v>
@@ -7581,16 +7597,16 @@
         <v>46225.616203564816</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I108" s="5">
         <v>46304</v>
@@ -7608,10 +7624,10 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P108" s="6" t="s">
         <v>26</v>
@@ -7624,7 +7640,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B109" s="9">
         <v>46225.60681763889</v>
@@ -7634,16 +7650,16 @@
         <v>46225.61619854167</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H109" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I109" s="9">
         <v>46304</v>
@@ -7661,10 +7677,10 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P109" s="10" t="s">
         <v>26</v>
@@ -7677,7 +7693,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B110" s="5">
         <v>46225.58153574074</v>
@@ -7687,7 +7703,7 @@
         <v>46225.60402078704</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>25</v>
@@ -7711,7 +7727,7 @@
         <v>26</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P110" s="6" t="s">
         <v>26</v>
@@ -7724,7 +7740,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B111" s="9">
         <v>46225.58153866898</v>
@@ -7734,16 +7750,16 @@
         <v>46225.61649424769</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F111" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G111" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="H111" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I111" s="9">
         <v>46307</v>
@@ -7761,13 +7777,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="O111" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Q111" s="9">
         <v>46311</v>
@@ -7787,7 +7803,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B112" s="5">
         <v>46225.58154590278</v>
@@ -7797,7 +7813,7 @@
         <v>46225.61639241898</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -7824,13 +7840,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Q112" s="5">
         <v>46311</v>
@@ -7850,7 +7866,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B113" s="9">
         <v>46225.59432256944</v>
@@ -7860,7 +7876,7 @@
         <v>46225.6052183912</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>25</v>
@@ -7884,7 +7900,7 @@
         <v>26</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="P113" s="10" t="s">
         <v>26</v>
@@ -7897,7 +7913,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B114" s="5">
         <v>46225.59476561342</v>
@@ -7907,7 +7923,7 @@
         <v>46225.616553796295</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
@@ -7934,13 +7950,13 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="Q114" s="5">
         <v>46318</v>
@@ -7960,7 +7976,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B115" s="9">
         <v>46225.59487494213</v>
@@ -7970,7 +7986,7 @@
         <v>46225.61655020833</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F115" s="10" t="s">
         <v>26</v>
@@ -7997,13 +8013,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O115" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="P115" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="Q115" s="9">
         <v>46325</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-09 22:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001580- CIA. RIO MINERALES.xlsx
+++ b/data/50001580- CIA. RIO MINERALES.xlsx
@@ -204,25 +204,22 @@
     <t>Alta</t>
   </si>
   <si>
+    <t>1216769310026544</t>
+  </si>
+  <si>
+    <t>Revision Tableros ot 4379</t>
+  </si>
+  <si>
+    <t>sergio saavedra fernandez</t>
+  </si>
+  <si>
+    <t>sergio.saavedra@zitron.com</t>
+  </si>
+  <si>
+    <t>ot  4379 -  TABLERO YD 63 KW,ot 4379 -  TABLERO YD 63 KW</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1216769310026544</t>
-  </si>
-  <si>
-    <t>Revision Tableros ot 4379</t>
-  </si>
-  <si>
-    <t>sergio saavedra fernandez</t>
-  </si>
-  <si>
-    <t>sergio.saavedra@zitron.com</t>
-  </si>
-  <si>
-    <t>ot  4379 -  TABLERO YD 63 KW,ot 4379 -  TABLERO YD 63 KW</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
   </si>
   <si>
     <t>1216769310026574</t>
@@ -360,6 +357,9 @@
   </si>
   <si>
     <t>Generacion oc tableros ot 4379</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
   </si>
   <si>
     <t>1216769310026536</t>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="9">
-        <v>46225.60046916667</v>
+        <v>46274.7341921412</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>45</v>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46231.20725755787</v>
+        <v>46274.73425525463</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2109,34 +2109,34 @@
         <v>52</v>
       </c>
       <c r="T10" s="6">
-        <v>0</v>
-      </c>
-      <c r="U10" s="12" t="s">
-        <v>53</v>
+        <v>1</v>
+      </c>
+      <c r="U10" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="9">
         <v>46225.58274704861</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="9">
-        <v>46225.61217166667</v>
+        <v>46274.73486938658</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I11" s="9">
         <v>46294</v>
@@ -2157,7 +2157,7 @@
         <v>45</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>45</v>
@@ -2172,15 +2172,15 @@
         <v>33</v>
       </c>
       <c r="T11" s="10">
-        <v>0</v>
-      </c>
-      <c r="U11" s="11" t="s">
-        <v>59</v>
+        <v>0.2</v>
+      </c>
+      <c r="U11" s="12" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12" s="5">
         <v>46225.59567834491</v>
@@ -2190,16 +2190,16 @@
         <v>46225.612248819445</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I12" s="5">
         <v>46294</v>
@@ -2217,13 +2217,13 @@
         <v>26</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="P12" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>63</v>
       </c>
       <c r="Q12" s="6"/>
       <c r="R12" s="6"/>
@@ -2233,7 +2233,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B13" s="9">
         <v>46225.595835520835</v>
@@ -2243,16 +2243,16 @@
         <v>46225.61224515046</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I13" s="9">
         <v>46294</v>
@@ -2270,13 +2270,13 @@
         <v>26</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O13" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="P13" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>63</v>
       </c>
       <c r="Q13" s="10"/>
       <c r="R13" s="10"/>
@@ -2286,7 +2286,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14" s="5">
         <v>46225.58085679398</v>
@@ -2298,7 +2298,7 @@
         <v>46226.576112442126</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>25</v>
@@ -2322,7 +2322,7 @@
         <v>26</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>26</v>
@@ -2339,7 +2339,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="9">
         <v>46225.58095215278</v>
@@ -2351,7 +2351,7 @@
         <v>46228.19449930555</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>26</v>
@@ -2372,19 +2372,19 @@
         <v>26</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>26</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="9">
         <v>46227</v>
@@ -2404,7 +2404,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46225.580861423616</v>
@@ -2414,7 +2414,7 @@
         <v>46225.59611458333</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>25</v>
@@ -2438,7 +2438,7 @@
         <v>26</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P16" s="6" t="s">
         <v>26</v>
@@ -2451,7 +2451,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B17" s="9">
         <v>46225.580958923616</v>
@@ -2461,16 +2461,16 @@
         <v>46237.5500087963</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I17" s="9">
         <v>46226</v>
@@ -2488,13 +2488,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="9">
         <v>46227</v>
@@ -2514,7 +2514,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="5">
         <v>46225.58096494213</v>
@@ -2524,16 +2524,16 @@
         <v>46237.550030706014</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I18" s="5">
         <v>46226</v>
@@ -2551,13 +2551,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>38</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q18" s="5">
         <v>46227</v>
@@ -2577,7 +2577,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9">
         <v>46225.58097109954</v>
@@ -2587,16 +2587,16 @@
         <v>46237.55005269676</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I19" s="9">
         <v>46226</v>
@@ -2614,13 +2614,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="9">
         <v>46227</v>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20" s="5">
         <v>46225.58086628473</v>
@@ -2650,7 +2650,7 @@
         <v>46225.59619578704</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>25</v>
@@ -2674,7 +2674,7 @@
         <v>26</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>26</v>
@@ -2687,7 +2687,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="9">
         <v>46225.580978240745</v>
@@ -2697,16 +2697,16 @@
         <v>46247.17789210648</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I21" s="9">
         <v>46245</v>
@@ -2724,13 +2724,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O21" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="P21" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="P21" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="Q21" s="9">
         <v>46246</v>
@@ -2745,12 +2745,12 @@
         <v>0</v>
       </c>
       <c r="U21" s="12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B22" s="5">
         <v>46225.5809840625</v>
@@ -2760,16 +2760,16 @@
         <v>46247.17788666667</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I22" s="5">
         <v>46245</v>
@@ -2787,13 +2787,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="Q22" s="5">
         <v>46246</v>
@@ -2808,12 +2808,12 @@
         <v>0</v>
       </c>
       <c r="U22" s="12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B23" s="9">
         <v>46225.58098827546</v>
@@ -2823,16 +2823,16 @@
         <v>46247.17788644676</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H23" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I23" s="9">
         <v>46245</v>
@@ -2850,13 +2850,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q23" s="9">
         <v>46246</v>
@@ -2871,12 +2871,12 @@
         <v>0</v>
       </c>
       <c r="U23" s="12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" s="5">
         <v>46225.58100011574</v>
@@ -2886,16 +2886,16 @@
         <v>46247.17788643518</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I24" s="5">
         <v>46245</v>
@@ -2913,13 +2913,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q24" s="5">
         <v>46246</v>
@@ -2934,12 +2934,12 @@
         <v>0</v>
       </c>
       <c r="U24" s="12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B25" s="9">
         <v>46225.59619364583</v>
@@ -2949,16 +2949,16 @@
         <v>46233.168979988426</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I25" s="9">
         <v>46231</v>
@@ -2976,13 +2976,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>48</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q25" s="9">
         <v>46232</v>
@@ -2997,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3107,7 +3107,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3152,7 +3152,7 @@
         <v>106</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>113</v>
@@ -3166,7 +3166,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3225,7 +3225,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3303,7 +3303,7 @@
         <v>46248.17134908565</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
@@ -3333,7 +3333,7 @@
         <v>118</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P31" s="10" t="s">
         <v>121</v>
@@ -3386,7 +3386,7 @@
         <v>118</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>124</v>
@@ -3457,7 +3457,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3472,7 +3472,7 @@
         <v>46248.17135226852</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
@@ -3502,7 +3502,7 @@
         <v>126</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P34" s="6" t="s">
         <v>129</v>
@@ -3555,7 +3555,7 @@
         <v>126</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>132</v>
@@ -3626,7 +3626,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -3848,7 +3848,7 @@
         <v>0</v>
       </c>
       <c r="U40" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -3863,7 +3863,7 @@
         <v>46241.17189372685</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
@@ -3893,7 +3893,7 @@
         <v>150</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P41" s="10" t="s">
         <v>155</v>
@@ -3946,7 +3946,7 @@
         <v>150</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>158</v>
@@ -4048,7 +4048,7 @@
         <v>160</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>166</v>
@@ -4148,7 +4148,7 @@
         <v>46245.1918381713</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
@@ -4259,7 +4259,7 @@
         <v>0</v>
       </c>
       <c r="U47" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -4475,7 +4475,7 @@
         <v>0</v>
       </c>
       <c r="U51" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -4538,7 +4538,7 @@
         <v>0</v>
       </c>
       <c r="U52" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -4601,7 +4601,7 @@
         <v>0</v>
       </c>
       <c r="U53" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4664,7 +4664,7 @@
         <v>0</v>
       </c>
       <c r="U54" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -4727,7 +4727,7 @@
         <v>0</v>
       </c>
       <c r="U55" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4790,7 +4790,7 @@
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4852,7 +4852,7 @@
         <v>46267.17196707176</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
@@ -4882,7 +4882,7 @@
         <v>207</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>212</v>
@@ -4900,7 +4900,7 @@
         <v>0</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -4963,7 +4963,7 @@
         <v>0</v>
       </c>
       <c r="U59" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5132,7 +5132,7 @@
         <v>0</v>
       </c>
       <c r="U62" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5326,7 +5326,7 @@
         <v>229</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>233</v>
@@ -5344,7 +5344,7 @@
         <v>0</v>
       </c>
       <c r="U66" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5389,7 +5389,7 @@
         <v>229</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P67" s="10" t="s">
         <v>236</v>
@@ -5407,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5452,7 +5452,7 @@
         <v>229</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>233</v>
@@ -5470,7 +5470,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5485,7 +5485,7 @@
         <v>46225.61467041667</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
@@ -5518,7 +5518,7 @@
         <v>157</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Q69" s="9">
         <v>46293</v>
@@ -5533,7 +5533,7 @@
         <v>0</v>
       </c>
       <c r="U69" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5601,10 +5601,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I71" s="9">
         <v>46275</v>
@@ -5643,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="U71" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5664,10 +5664,10 @@
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I72" s="5">
         <v>46275</v>
@@ -5717,10 +5717,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I73" s="9">
         <v>46275</v>
@@ -5770,10 +5770,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I74" s="5">
         <v>46286</v>
@@ -5812,7 +5812,7 @@
         <v>0</v>
       </c>
       <c r="U74" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5833,10 +5833,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I75" s="9">
         <v>46286</v>
@@ -5886,10 +5886,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I76" s="5">
         <v>46286</v>
@@ -5939,10 +5939,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I77" s="9">
         <v>46287</v>
@@ -5981,7 +5981,7 @@
         <v>0</v>
       </c>
       <c r="U77" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6002,10 +6002,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="5">
@@ -6053,10 +6053,10 @@
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H79" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6104,10 +6104,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I80" s="5">
         <v>46288</v>
@@ -6146,7 +6146,7 @@
         <v>0</v>
       </c>
       <c r="U80" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6167,10 +6167,10 @@
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H81" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H81" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I81" s="9">
         <v>46288</v>
@@ -6220,10 +6220,10 @@
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I82" s="5">
         <v>46288</v>
@@ -6273,10 +6273,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H83" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H83" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I83" s="9">
         <v>46289</v>
@@ -6326,10 +6326,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H84" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I84" s="5">
         <v>46290</v>
@@ -6368,7 +6368,7 @@
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6389,10 +6389,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H85" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H85" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="9">
@@ -6440,10 +6440,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="5">
@@ -6491,10 +6491,10 @@
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H87" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H87" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I87" s="9">
         <v>46293</v>
@@ -6533,7 +6533,7 @@
         <v>0</v>
       </c>
       <c r="U87" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -6554,10 +6554,10 @@
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H88" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H88" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I88" s="5">
         <v>46293</v>
@@ -6607,10 +6607,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H89" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H89" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I89" s="9">
         <v>46293</v>
@@ -6749,7 +6749,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -6896,7 +6896,7 @@
         <v>294</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P94" s="6" t="s">
         <v>304</v>
@@ -6947,7 +6947,7 @@
         <v>294</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P95" s="10" t="s">
         <v>304</v>
@@ -6976,10 +6976,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="5">
@@ -7016,7 +7016,7 @@
         <v>0</v>
       </c>
       <c r="U96" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -7037,10 +7037,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H97" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H97" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I97" s="9">
         <v>46302</v>
@@ -7090,10 +7090,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H98" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I98" s="5">
         <v>46302</v>
@@ -7143,10 +7143,10 @@
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H99" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="H99" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="I99" s="9">
         <v>46302</v>
@@ -7196,10 +7196,10 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H100" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="H100" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="I100" s="5">
         <v>46302</v>
@@ -7291,7 +7291,7 @@
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -7562,7 +7562,7 @@
         <v>0</v>
       </c>
       <c r="U106" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
@@ -7880,7 +7880,7 @@
         <v>0</v>
       </c>
       <c r="U112" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
@@ -7943,7 +7943,7 @@
         <v>0</v>
       </c>
       <c r="U113" s="11" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>